<commit_message>
done more changes related to the new instance of cis lms
</commit_message>
<xml_diff>
--- a/public/sample-files/user-upload-sample-file.xlsx
+++ b/public/sample-files/user-upload-sample-file.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20361"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lms\public\sample-files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Q276\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641C5D8B-32EC-461A-99AD-A750B121FFDD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9ABD779-C0E2-440B-92FD-BD43D213AF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="8505" xr2:uid="{A7F8B422-7AB2-4EBC-9E52-5BE7BFC3BBDD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{2A36A1C1-3867-466B-8916-67C33ECE06DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>SL No.</t>
   </si>
@@ -48,13 +48,7 @@
     <t>Designation*</t>
   </si>
   <si>
-    <t>LOB</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Circle</t>
+    <t>Agency</t>
   </si>
   <si>
     <t>Gender*</t>
@@ -94,7 +88,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,12 +128,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -209,7 +197,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -226,22 +214,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -561,11 +543,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C534C55-876D-4955-9411-F2322915B4B9}">
-  <dimension ref="A1:K3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E4162E-40F6-4963-96A9-F885315B1231}">
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,78 +583,68 @@
       <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>13</v>
       </c>
       <c r="F2" s="6">
         <v>9876543217</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="6" t="s">
-        <v>15</v>
+      <c r="G2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="9"/>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="E3" s="8" t="s">
         <v>17</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>19</v>
       </c>
       <c r="F3" s="6">
         <v>2345678987</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="6" t="s">
-        <v>15</v>
+      <c r="G3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{14D300C0-41A2-4425-8933-05A6F74B7379}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{7CD364CF-BFD1-470F-8261-29F2535831AF}"/>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{CBF15E6A-F769-429B-9C16-F5B3D5CEE3B3}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{6F06883C-D2CE-4C0B-B666-D560962E9157}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>